<commit_message>
Update README with full documentation, update CLAUDE.md and Excel template
- README: complete rewrite with installation, usage, CLI args, Excel format,
  payment types, output structure, business rules overview, project structure
- CLAUDE.md: update status to Phase 1 implemented, add domain knowledge
  (QRR as Prtry, validation against transaction data, charset rules)
- Excel template: expand to 10 test cases including SEPA with overrides
  and CBPR+ JPY payment

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/testfaelle_vorlage.xlsx
+++ b/templates/testfaelle_vorlage.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -560,7 +560,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Negative SEPA-Zahlung mit falscher Waehrung</t>
+          <t>Negative SEPA-Zahlung: Waehrung wird auf CHF gesetzt</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -595,24 +595,24 @@
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Waehrung wird auf CHF gesetzt</t>
+          <t>Erwartet: BR-SEPA-001 verletzt (Waehrung != EUR)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TC-QR-001</t>
+          <t>TC-SEPA-003</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>QR-Zahlung Standard</t>
+          <t>SEPA mit Creditor-Override</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Positive QR-Zahlung mit QR-IBAN und QRR</t>
+          <t>SEPA-Zahlung mit explizitem Creditor-Namen und BIC</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -622,15 +622,15 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Domestic-QR</t>
+          <t>SEPA</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3200</v>
+        <v>4999.99</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>CHF</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -638,30 +638,38 @@
           <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Cdtr.Nm=Beispiel GmbH; CdtrAgt.BICFI=COBADEFFXXX</t>
+        </is>
+      </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Creditor wird explizit gesetzt statt generiert</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TC-QR-002</t>
+          <t>TC-QR-001</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>QR-Zahlung ohne Referenz</t>
+          <t>QR-Zahlung Standard CHF</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Negative QR-Zahlung ohne QRR-Referenz</t>
+          <t>Positive QR-Zahlung mit QR-IBAN und QRR</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -670,7 +678,7 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>890</v>
+        <v>3200</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -682,47 +690,39 @@
           <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>ViolateRule=BR-QR-002</t>
-        </is>
-      </c>
+      <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>QRR-Referenz wird entfernt</t>
-        </is>
-      </c>
+      <c r="L5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TC-IBAN-001</t>
+          <t>TC-QR-002</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Domestic IBAN Standard</t>
+          <t>QR-Zahlung ohne Referenz</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Positive Inlandszahlung mit regulaerer IBAN</t>
+          <t>Negative QR-Zahlung: QRR-Referenz wird entfernt</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Domestic-IBAN</t>
+          <t>Domestic-QR</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>5000</v>
+        <v>890</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -734,30 +734,38 @@
           <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>ViolateRule=BR-QR-002</t>
+        </is>
+      </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Erwartet: BR-QR-002 verletzt (keine QRR bei QR-IBAN)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TC-IBAN-002</t>
+          <t>TC-IBAN-001</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Domestic IBAN falsche Waehrung</t>
+          <t>Domestic IBAN Standard</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Negative Inlandszahlung mit EUR statt CHF</t>
+          <t>Positive Inlandszahlung mit regulaerer CH-IBAN</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -766,7 +774,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>750</v>
+        <v>5000</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -778,51 +786,43 @@
           <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>ViolateRule=BR-IBAN-004</t>
-        </is>
-      </c>
+      <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>Waehrung wird auf EUR gesetzt</t>
-        </is>
-      </c>
+      <c r="L7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TC-CBPR-001</t>
+          <t>TC-IBAN-002</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CBPR+ Standardzahlung</t>
+          <t>Domestic IBAN falsche Waehrung</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Positive Cross-Border-Zahlung</t>
+          <t>Negative Inlandszahlung: Waehrung wird auf EUR gesetzt</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>CBPR+</t>
+          <t>Domestic-IBAN</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>10000</v>
+        <v>750</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>CHF</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -832,32 +832,36 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>CdtrAgt.BICFI=BNPAFRPP</t>
+          <t>ViolateRule=BR-IBAN-004</t>
         </is>
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Erwartet: BR-IBAN-004 verletzt (Waehrung != CHF)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TC-CBPR-002</t>
+          <t>TC-CBPR-001</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CBPR+ ohne Agent</t>
+          <t>CBPR+ USD-Zahlung</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Negative CBPR+ ohne Creditor-Agent</t>
+          <t>Positive Cross-Border-Zahlung in USD</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -866,11 +870,11 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2500</v>
+        <v>10000</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -880,14 +884,114 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>CdtrAgt.BICFI=BARCGB22; ViolateRule=BR-CBPR-005</t>
+          <t>CdtrAgt.BICFI=BNPAFRPP</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>Creditor-Agent BIC wird entfernt</t>
+      <c r="L9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>TC-CBPR-002</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>CBPR+ ohne Agent</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Negative CBPR+: Creditor-Agent BIC wird entfernt</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>CBPR+</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>2500</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>CdtrAgt.BICFI=BARCGB22; ViolateRule=BR-CBPR-005</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Erwartet: BR-CBPR-005 verletzt (kein Creditor-Agent)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TC-CBPR-003</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>CBPR+ JPY-Zahlung</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Positive Cross-Border-Zahlung in JPY</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>CBPR+</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>500000</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>CdtrAgt.BICFI=BOABORJ1</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Japanische Yen-Zahlung</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 10 multi-payment test cases and regenerate examples
New test cases TC-MULTI-001 through TC-MULTI-010:
- 6 single-PmtInf with TxCount 2-3 (SEPA, QR, IBAN, CBPR+)
  - 2 NOK cases: BR-SEPA-004 (name too long), BR-QR-003 (SCOR on QR)
- 2 multi-PmtInf groups (BATCH-A, BATCH-B), each with 2 PmtInf
  and TxCount=2 per PmtInf, mixing payment types

All 20 test cases pass. Multi-payment XMLs XSD-validated:
- BATCH-A: 2 PmtInf (SEPA+IBAN), 4 transactions, CtrlSum=13000
- BATCH-B: 2 PmtInf (CBPR++SEPA), 4 transactions, CtrlSum=32500

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/testfaelle_vorlage.xlsx
+++ b/templates/testfaelle_vorlage.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -542,10 +542,6 @@
           <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -591,8 +587,6 @@
           <t>ViolateRule=BR-SEPA-001</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
           <t>Erwartet: BR-SEPA-001 verletzt (Waehrung != EUR)</t>
@@ -643,8 +637,6 @@
           <t>Cdtr.Nm=Beispiel GmbH; CdtrAgt.BICFI=COBADEFFXXX</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
           <t>Creditor wird explizit gesetzt statt generiert</t>
@@ -690,10 +682,6 @@
           <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -739,8 +727,6 @@
           <t>ViolateRule=BR-QR-002</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
           <t>Erwartet: BR-QR-002 verletzt (keine QRR bei QR-IBAN)</t>
@@ -786,10 +772,6 @@
           <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -835,8 +817,6 @@
           <t>ViolateRule=BR-IBAN-004</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
           <t>Erwartet: BR-IBAN-004 verletzt (Waehrung != CHF)</t>
@@ -887,9 +867,6 @@
           <t>CdtrAgt.BICFI=BNPAFRPP</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -935,8 +912,6 @@
           <t>CdtrAgt.BICFI=BARCGB22; ViolateRule=BR-CBPR-005</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
           <t>Erwartet: BR-CBPR-005 verletzt (kein Creditor-Agent)</t>
@@ -987,11 +962,509 @@
           <t>CdtrAgt.BICFI=BOABORJ1</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
           <t>Japanische Yen-Zahlung</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>TC-MULTI-001</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>SEPA Sammelzahlung 3 Tx</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>SEPA mit 3 Transaktionen in einem PmtInf</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>SEPA</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>750</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>TxCount=3</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>1 B-Level, 3 C-Levels</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>TC-MULTI-002</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>QR-Sammelzahlung 2 Tx</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Domestic-QR mit 2 Transaktionen in einem PmtInf</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Domestic-QR</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>1200</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>TxCount=2</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>1 B-Level, 2 C-Levels</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>TC-MULTI-003</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Domestic-IBAN Sammelzahlung 2 Tx</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Domestic-IBAN mit 2 Transaktionen</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Domestic-IBAN</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>3500</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>TxCount=2</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>1 B-Level, 2 C-Levels</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>TC-MULTI-004</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>CBPR+ Sammelzahlung 2 Tx</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>CBPR+ mit 2 Transaktionen und explizitem BIC</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>CBPR+</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>8000</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>TxCount=2; CdtrAgt.BICFI=CHASUS33</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>1 B-Level, 2 C-Levels</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>TC-MULTI-005</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>SEPA Sammelzahlung NOK Name</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>SEPA TxCount=2 mit zu langem Creditor-Namen</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>SEPA</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>500</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>TxCount=2; ViolateRule=BR-SEPA-004</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Erwartet: BR-SEPA-004 verletzt bei allen Tx</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>TC-MULTI-006</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>QR-Sammelzahlung NOK SCOR</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>QR TxCount=2 mit unzulaessiger SCOR-Referenz</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Domestic-QR</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>990</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>TxCount=2; ViolateRule=BR-QR-003</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Erwartet: BR-QR-003 verletzt (SCOR bei QR-IBAN)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>TC-MULTI-007</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Batch-A: SEPA-Teil</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Multi-Payment BATCH-A: SEPA mit 2 Tx</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>SEPA</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>GroupId=BATCH-A; TxCount=2</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Gruppe BATCH-A, PmtInf 1 von 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>TC-MULTI-008</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Batch-A: Domestic-IBAN-Teil</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Multi-Payment BATCH-A: Domestic-IBAN mit 2 Tx</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Domestic-IBAN</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>4500</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>GroupId=BATCH-A; TxCount=2</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Gruppe BATCH-A, PmtInf 2 von 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>TC-MULTI-009</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Batch-B: CBPR+-Teil</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Multi-Payment BATCH-B: CBPR+ mit 2 Tx</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>CBPR+</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>15000</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>GroupId=BATCH-B; TxCount=2; CdtrAgt.BICFI=BNPAFRPP</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Gruppe BATCH-B, PmtInf 1 von 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>TC-MULTI-010</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Batch-B: SEPA-Teil</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Multi-Payment BATCH-B: SEPA mit 2 Tx</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>SEPA</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>1250</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>GroupId=BATCH-B; TxCount=2</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Gruppe BATCH-B, PmtInf 2 von 2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 25 comprehensive test cases, fix BR-SEPA-003 validation and DbtrAgt
New test cases (45 total):
- All remaining violatable rules: BR-SEPA-003, BR-QR-004, BR-IBAN-001,
  BR-IBAN-002 (BR-CBPR-001 skipped, validation checks testcase not tx)
- SEPA edge cases: min/max amounts, 70-char name boundary, full overrides
- QR: EUR variant, min amount
- Domestic-IBAN: min/max amounts
- CBPR+: EUR, GBP, CHF currencies
- Debtor variants: minimal (no BIC/address), alternative company
- 3-way multi-payment group (BATCH-C: SEPA+QR+IBAN)
- Mixed OK/NOK multi-payment group (BATCH-D)

Bug fixes:
- Add BR-SEPA-003 validation (ChrgBr must be SLEV) — was violatable
  but never checked
- Fix DbtrAgt without BIC: remove invalid Othr/NOTPROVIDED, use empty
  FinInstnId instead (SPS XSD allows all fields optional)

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/testfaelle_vorlage.xlsx
+++ b/templates/testfaelle_vorlage.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1468,6 +1468,1206 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>TC-SEPA-004</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>SEPA falsche Gebuehrenregelung</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Negative SEPA: ChrgBr wird auf DEBT statt SLEV gesetzt</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>SEPA</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>ViolateRule=BR-SEPA-003</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Erwartet: BR-SEPA-003 verletzt (ChrgBr != SLEV)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>TC-SEPA-005</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>SEPA zu langer Creditor-Name</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Negative SEPA: Creditor-Name wird auf 71 Zeichen gesetzt</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>SEPA</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>800</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>ViolateRule=BR-SEPA-004</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Erwartet: BR-SEPA-004 verletzt (Name &gt; 70 Zeichen)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>TC-QR-003</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>QR-Zahlung falsche Waehrung</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Negative QR: Waehrung wird auf USD gesetzt (nur CHF/EUR erlaubt)</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Domestic-QR</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>1500</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>ViolateRule=BR-QR-004</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Erwartet: BR-QR-004 verletzt (Waehrung nicht CHF/EUR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>TC-IBAN-003</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Domestic-IBAN mit QR-IBAN</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Negative IBAN: QR-IBAN wird als Creditor gesetzt</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Domestic-IBAN</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>ViolateRule=BR-IBAN-001</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Erwartet: BR-IBAN-001 verletzt (QR-IBAN statt regulaere)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>TC-IBAN-005</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Domestic-IBAN mit QRR-Referenz</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Negative IBAN: QRR-Referenz bei regulaerer IBAN</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Domestic-IBAN</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>1800</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>ViolateRule=BR-IBAN-002</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Erwartet: BR-IBAN-002 verletzt (QRR bei regulaerer IBAN)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>TC-SEPA-006</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>SEPA Kleinstbetrag</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>SEPA mit Minimalbetrag 0.01 EUR</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>SEPA</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>Grenzwert: kleinster zulaessiger Betrag</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>TC-SEPA-007</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>SEPA Grossbetrag</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>SEPA nahe am Betragslimit (999999.99 EUR)</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>SEPA</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>999999.99</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>Hoher Betrag, innerhalb SEPA-Limit</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>TC-SEPA-008</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>SEPA Grenzwert Creditor-Name 70 Zeichen</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>SEPA mit Creditor-Name genau 70 Zeichen (Grenzwert)</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>SEPA</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>500</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Cdtr.Nm=AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>Grenzwert: exakt 70 Zeichen, muss OK sein</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>TC-SEPA-009</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>SEPA mit vollem Creditor-Override</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>SEPA mit explizitem Creditor-Namen, BIC und Adresse</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>SEPA</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Cdtr.Nm=Deutsche Bank AG; CdtrAgt.BICFI=DEUTDEFF</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>Alle Creditor-Felder uebersteuert</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>TC-SEPA-010</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>SEPA SEPA-Maxbetrag</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>SEPA mit absolutem Maximum 999999999.99 EUR</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>SEPA</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>999999999.99</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>Grenzwert: SEPA-Maximum (BR-SEPA-006)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>TC-QR-004</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>QR-Zahlung EUR</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Positive QR-Zahlung in EUR (CHF und EUR erlaubt)</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Domestic-QR</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>750</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>QR-IBAN mit EUR statt CHF</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>TC-QR-005</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>QR-Zahlung Kleinstbetrag</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>QR-Zahlung mit Minimalbetrag</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Domestic-QR</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>Grenzwert: kleinster zulaessiger Betrag</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>TC-IBAN-006</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Domestic-IBAN Kleinstbetrag</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Inlandszahlung mit Minimalbetrag</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Domestic-IBAN</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>Kleiner CHF-Betrag</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>TC-IBAN-007</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Domestic-IBAN Grossbetrag</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Inlandszahlung mit hohem Betrag</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Domestic-IBAN</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>500000</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>Grossbetrag Inland</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>TC-CBPR-004</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>CBPR+ EUR-Zahlung</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Cross-Border in EUR mit deutschem BIC</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>CBPR+</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>25000</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>CdtrAgt.BICFI=DEUTDEFF</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>CBPR+ mit europaeischer Waehrung</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>TC-CBPR-005</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>CBPR+ GBP-Zahlung</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Cross-Border in GBP mit britischem BIC</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>CBPR+</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>8500</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>CdtrAgt.BICFI=BARCGB22</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>CBPR+ Pfund Sterling</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>TC-CBPR-006</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>CBPR+ CHF-Zahlung</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Cross-Border in CHF (auch bei CBPR+ moeglich)</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>CBPR+</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>12000</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>CdtrAgt.BICFI=UBSWCHZH80A</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>CBPR+ mit Schweizer Franken</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>TC-DBT-001</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Minimaler Debtor</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>SEPA-Zahlung mit minimalem Debtor (nur Name und IBAN)</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>SEPA</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>200</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Name=Klein GmbH; IBAN=CH9300762011623852957</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>Debtor ohne BIC, Adresse — NOTPROVIDED im XML</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>TC-DBT-002</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Alternativer Debtor</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>QR-Zahlung mit anderem Debtor-Konto</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Domestic-QR</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>4200</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Name=Helvetia Versicherungen AG; IBAN=CH3908704016075473007; BIC=RAIFCH22; Strasse=Dufourstrasse; Hausnummer=40; PLZ=9001; Ort=St. Gallen; Land=CH</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>Anderer Debtor (Helvetia)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>TC-DBT-003</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Alternativer Debtor Domestic</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Domestic-IBAN mit alternativem Debtor</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Domestic-IBAN</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>9500</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Name=Helvetia Versicherungen AG; IBAN=CH3908704016075473007; BIC=RAIFCH22; Strasse=Dufourstrasse; Hausnummer=40; PLZ=9001; Ort=St. Gallen; Land=CH</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Helvetia als Debtor bei Inlandszahlung</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>TC-BATCH-C-001</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Batch-C: SEPA-Teil</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Multi-Payment 3er-Gruppe: SEPA</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>SEPA</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>1500</v>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>GroupId=BATCH-C</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>Gruppe BATCH-C: PmtInf 1 von 3 (SEPA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>TC-BATCH-C-002</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Batch-C: QR-Teil</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Multi-Payment 3er-Gruppe: QR</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Domestic-QR</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>2200</v>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>GroupId=BATCH-C</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>Gruppe BATCH-C: PmtInf 2 von 3 (QR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>TC-BATCH-C-003</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Batch-C: IBAN-Teil</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Multi-Payment 3er-Gruppe: Domestic-IBAN</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Domestic-IBAN</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>3300</v>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>GroupId=BATCH-C</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>Gruppe BATCH-C: PmtInf 3 von 3 (IBAN)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>TC-BATCH-D-001</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Batch-D: SEPA OK-Teil</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Multi-Payment gemischt: SEPA korrekt</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>SEPA</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>600</v>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>GroupId=BATCH-D</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>Gruppe BATCH-D: OK-Anteil</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>TC-BATCH-D-002</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Batch-D: SEPA NOK-Teil</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Multi-Payment gemischt: SEPA falsche Waehrung</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>SEPA</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>400</v>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>GroupId=BATCH-D; ViolateRule=BR-SEPA-001</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>Gruppe BATCH-D: NOK-Anteil (Waehrung verletzt)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 10 NOK test cases, fix BR-CBPR-001 validation
New NOK test cases (55 total):
- Violations with TxCount>1: BR-SEPA-001 (3 Tx), BR-QR-002 (3 Tx),
  BR-IBAN-001 (2 Tx), BR-IBAN-002 (2 Tx), BR-CBPR-005 (2 Tx)
- Violations with alternative debtor: BR-SEPA-003, BR-QR-004
- Multi-payment group BATCH-E with mixed OK/NOK (3 members)

Fixes:
- Fix BR-CBPR-001 validation: check transaction currency instead of
  testcase currency (matches how violations modify data)
- Mark BR-CBPR-001 as non-violatable: empty currency breaks XSD
  (Ccy attribute requires 3-letter pattern), this is an input-level
  check not testable via XML violation

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/testfaelle_vorlage.xlsx
+++ b/templates/testfaelle_vorlage.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L46"/>
+  <dimension ref="A1:L56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -2668,6 +2668,506 @@
         </is>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>TC-NOK-001</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>SEPA 3 Tx falsche Waehrung</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>SEPA TxCount=3: alle Tx bekommen CHF statt EUR</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>SEPA</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>TxCount=3; ViolateRule=BR-SEPA-001</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>BR-SEPA-001 bei allen 3 Transaktionen</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>TC-NOK-002</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>QR 3 Tx ohne Referenz</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>QR TxCount=3: QRR-Referenz wird bei allen Tx entfernt</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Domestic-QR</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v>800</v>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>TxCount=3; ViolateRule=BR-QR-002</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>BR-QR-002 bei allen 3 Transaktionen</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>TC-NOK-003</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>IBAN 2 Tx mit QR-IBAN</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>IBAN TxCount=2: QR-IBAN statt regulaere IBAN</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Domestic-IBAN</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>2500</v>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>TxCount=2; ViolateRule=BR-IBAN-001</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>BR-IBAN-001 bei 2 Transaktionen</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>TC-NOK-004</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>CBPR+ 2 Tx ohne Agent</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>CBPR+ TxCount=2: Creditor-Agent BIC entfernt</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>CBPR+</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>7500</v>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>TxCount=2; CdtrAgt.BICFI=BARCGB22; ViolateRule=BR-CBPR-005</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>BR-CBPR-005 bei 2 Transaktionen</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>TC-NOK-005</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>IBAN 2 Tx mit QRR</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>IBAN TxCount=2: QRR-Referenz bei regulaerer IBAN</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Domestic-IBAN</t>
+        </is>
+      </c>
+      <c r="F51" t="n">
+        <v>1200</v>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>TxCount=2; ViolateRule=BR-IBAN-002</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>BR-IBAN-002 bei 2 Transaktionen</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>TC-BATCH-E-001</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Batch-E: SEPA OK</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Multi-Payment gemischt: SEPA korrekt</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>SEPA</t>
+        </is>
+      </c>
+      <c r="F52" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>GroupId=BATCH-E; TxCount=2</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>Gruppe BATCH-E: OK-Teil</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>TC-BATCH-E-002</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Batch-E: QR NOK ohne Ref</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Multi-Payment gemischt: QR-Referenz entfernt</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Domestic-QR</t>
+        </is>
+      </c>
+      <c r="F53" t="n">
+        <v>1500</v>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>GroupId=BATCH-E; ViolateRule=BR-QR-002</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>Gruppe BATCH-E: NOK-Teil (BR-QR-002)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>TC-BATCH-E-003</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Batch-E: CBPR+ NOK ohne BIC</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Multi-Payment gemischt: Agent-BIC entfernt</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>CBPR+</t>
+        </is>
+      </c>
+      <c r="F54" t="n">
+        <v>9000</v>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>GroupId=BATCH-E; CdtrAgt.BICFI=CHASUS33; ViolateRule=BR-CBPR-005</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>Gruppe BATCH-E: NOK-Teil (BR-CBPR-005)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>TC-NOK-007</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>SEPA falsche Gebuehr anderer Debtor</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>SEPA mit Helvetia-Debtor: ChrgBr=DEBT</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>SEPA</t>
+        </is>
+      </c>
+      <c r="F55" t="n">
+        <v>5500</v>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Name=Helvetia Versicherungen AG; IBAN=CH3908704016075473007; BIC=RAIFCH22; Strasse=Dufourstrasse; Hausnummer=40; PLZ=9001; Ort=St. Gallen; Land=CH</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>ViolateRule=BR-SEPA-003</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>BR-SEPA-003 mit alternativem Debtor</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>TC-NOK-008</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>QR falsche Waehrung anderer Debtor</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>QR mit Helvetia-Debtor: USD statt CHF/EUR</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Domestic-QR</t>
+        </is>
+      </c>
+      <c r="F56" t="n">
+        <v>3200</v>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Name=Helvetia Versicherungen AG; IBAN=CH3908704016075473007; BIC=RAIFCH22; Strasse=Dufourstrasse; Hausnummer=40; PLZ=9001; Ort=St. Gallen; Land=CH</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>ViolateRule=BR-QR-004</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>BR-QR-004 mit alternativem Debtor</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 8 new business rules from SwissQRBill analysis + SPS specs
New rules (36 total):
- BR-GEN-001: Amount max 2 decimal places (SPS 2025 §2.5)
- BR-GEN-002: BIC format 8 or 11 alphanumeric chars (IG CT §3.12)
- BR-GEN-006: Creditor name max 140 chars for non-SEPA (IG CT v2.2)
- BR-GEN-007: Country code must be 2 uppercase letters (ISO 3166-1)
- BR-ADDR-001: Structured address: TwnNm + Ctry mandatory (SPS §3.11)
- BR-QR-007: QR-IBAN must be CH or LI (SwissQRBill + SPS)
- BR-IBAN-006: Domestic IBAN must be CH or LI (SwissQRBill + SPS)
- BR-REF-V01: SCOR format RF + check digits, max 25 chars (ISO 11649)

New categories in catalog: ADDR (address rules), REF-V (reference validation)
10 new test cases (TC-VAL-001 to TC-VAL-010), 65 total, all passing.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/testfaelle_vorlage.xlsx
+++ b/templates/testfaelle_vorlage.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L56"/>
+  <dimension ref="A1:L66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -3168,6 +3168,471 @@
         </is>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>TC-VAL-001</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Betrag mit 2 Dezimalstellen</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Betrag 123.45 hat genau 2 Dezimalstellen (OK)</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>SEPA</t>
+        </is>
+      </c>
+      <c r="F57" t="n">
+        <v>123.45</v>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>BR-GEN-001: exakt 2 Dezimalstellen</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>TC-VAL-002</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>BIC 8 Zeichen</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Creditor-BIC mit 8 Zeichen (OK)</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>CBPR+</t>
+        </is>
+      </c>
+      <c r="F58" t="n">
+        <v>5000</v>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>CdtrAgt.BICFI=BNPAFRPP</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>BR-GEN-002: 8-stelliger BIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>TC-VAL-003</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>BIC 11 Zeichen</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Creditor-BIC mit 11 Zeichen (OK)</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>CBPR+</t>
+        </is>
+      </c>
+      <c r="F59" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>CdtrAgt.BICFI=BARCGB22XXX</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>BR-GEN-002: 11-stelliger BIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>TC-VAL-004</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Country-Code DE</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>SEPA mit deutschem Creditor-Country (OK)</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>SEPA</t>
+        </is>
+      </c>
+      <c r="F60" t="n">
+        <v>750</v>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>BR-GEN-007: gültiger Country-Code DE</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>TC-VAL-005</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Vollstaendige Creditor-Adresse</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Creditor mit vollstaendiger strukturierter Adresse (OK)</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Domestic-IBAN</t>
+        </is>
+      </c>
+      <c r="F61" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>BR-ADDR-001: TwnNm und Ctry vorhanden</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>TC-VAL-006</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Creditor-Name 140 Zeichen non-SEPA</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Domestic-IBAN mit 140-Zeichen-Creditor-Name (Grenzwert)</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Domestic-IBAN</t>
+        </is>
+      </c>
+      <c r="F62" t="n">
+        <v>1500</v>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Cdtr.Nm=BBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBBB</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>BR-GEN-006: exakt 140 Zeichen, muss OK sein</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>TC-VAL-007</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>QR-IBAN CH-Laenderkennzeichen</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>QR-Zahlung mit CH-QR-IBAN (OK)</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Domestic-QR</t>
+        </is>
+      </c>
+      <c r="F63" t="n">
+        <v>900</v>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>BR-QR-007: CH-IBAN korrekt</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>TC-VAL-008</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Domestic-IBAN CH-Laenderkennzeichen</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Inlandszahlung mit CH-IBAN (OK)</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Domestic-IBAN</t>
+        </is>
+      </c>
+      <c r="F64" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>BR-IBAN-006: CH-IBAN korrekt</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>TC-VAL-009</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>SCOR-Referenz valide</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Domestic-IBAN mit generierter SCOR-Referenz (OK)</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Domestic-IBAN</t>
+        </is>
+      </c>
+      <c r="F65" t="n">
+        <v>800</v>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>BR-REF-V01: generierte SCOR ist valide</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>TC-VAL-010</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Betrag ganzzahlig</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>SEPA mit ganzzahligem Betrag 1000 (OK)</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>SEPA</t>
+        </is>
+      </c>
+      <c r="F66" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Name=Muster AG; IBAN=CH5604835012345678009; BIC=CRESCHZZ80A; Strasse=Bahnhofstrasse; Hausnummer=1; PLZ=8001; Ort=Zuerich; Land=CH</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>BR-GEN-001: 0 Dezimalstellen ist OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>